<commit_message>
Regenerate demo data Excel files
https://claude.ai/code/session_01TN2hEKgdHt2r7RfJDisQSu
</commit_message>
<xml_diff>
--- a/demo_data/appointments.xlsx
+++ b/demo_data/appointments.xlsx
@@ -471,44 +471,40 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>UHID-1002</t>
+          <t>UHID-1007</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Dr. Manish Gupta</t>
+          <t>Dr. Kavita Nair</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Paediatrics</t>
+          <t>Pulmonology</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>booked</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>OPD</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Medication review</t>
-        </is>
-      </c>
+          <t>Follow-up</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -518,12 +514,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>UHID-1018</t>
+          <t>UHID-1008</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Dr. Suresh Reddy</t>
+          <t>Dr. Priya Mehta</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -533,29 +529,25 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>booked</t>
+          <t>cancelled</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Procedure</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Routine check-up</t>
-        </is>
-      </c>
+          <t>Follow-up</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -565,44 +557,40 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>UHID-1015</t>
+          <t>UHID-1006</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Dr. Kavita Nair</t>
+          <t>Dr. Priya Mehta</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Gastroenterology</t>
+          <t>Psychiatry</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>booked</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Post-surgery review</t>
-        </is>
-      </c>
+          <t>OPD</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -612,42 +600,42 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>UHID-1019</t>
+          <t>UHID-1008</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Dr. Arjun Verma</t>
+          <t>Dr. Deepa Iyer</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Gastroenterology</t>
+          <t>Paediatrics</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>cancelled</t>
+          <t>booked</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Review</t>
+          <t>OPD</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Routine check-up</t>
+          <t>Medication review</t>
         </is>
       </c>
     </row>
@@ -659,7 +647,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>UHID-1013</t>
+          <t>UHID-1002</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -669,34 +657,30 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Neurology</t>
+          <t>Pulmonology</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>booked</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Follow-up</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Routine check-up</t>
-        </is>
-      </c>
+          <t>Procedure</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -706,27 +690,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>UHID-1011</t>
+          <t>UHID-1007</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Dr. Deepa Iyer</t>
+          <t>Dr. Kavita Nair</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Paediatrics</t>
+          <t>Psychiatry</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -736,14 +720,10 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>OPD</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Routine check-up</t>
-        </is>
-      </c>
+          <t>Follow-up</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -753,32 +733,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>UHID-1002</t>
+          <t>UHID-1014</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Dr. Priya Mehta</t>
+          <t>Dr. Manish Gupta</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Psychiatry</t>
+          <t>Neurology</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12:45</t>
+          <t>10:15</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>booked</t>
+          <t>cancelled</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -800,40 +780,44 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>UHID-1013</t>
+          <t>UHID-1001</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Dr. Vikram Rao</t>
+          <t>Dr. Priya Mehta</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Pulmonology</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>booked</t>
+          <t>cancelled</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Procedure</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr"/>
+          <t>OPD</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Routine check-up</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -843,7 +827,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>UHID-1010</t>
+          <t>UHID-1000</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -853,27 +837,27 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Psychiatry</t>
+          <t>Oncology</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>cancelled</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>OPD</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -890,27 +874,27 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>UHID-1012</t>
+          <t>UHID-1016</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Dr. Sunita Sharma</t>
+          <t>Dr. Rajesh Kumar</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Psychiatry</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -920,10 +904,14 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>OPD</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr"/>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Routine check-up</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -933,37 +921,37 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>UHID-1010</t>
+          <t>UHID-1000</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Dr. Sunita Sharma</t>
+          <t>Dr. Vikram Rao</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Gynaecology</t>
+          <t>Orthopaedics</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>booked</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>OPD</t>
+          <t>Procedure</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -980,27 +968,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>UHID-1010</t>
+          <t>UHID-1009</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Dr. Arjun Verma</t>
+          <t>Dr. Sunita Sharma</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Paediatrics</t>
+          <t>Orthopaedics</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>13:45</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1010,14 +998,10 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Routine check-up</t>
-        </is>
-      </c>
+          <t>Procedure</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1027,12 +1011,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>UHID-1019</t>
+          <t>UHID-1008</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Dr. Priya Mehta</t>
+          <t>Dr. Suresh Reddy</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1042,12 +1026,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1062,7 +1046,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Post-surgery review</t>
+          <t>Medication review</t>
         </is>
       </c>
     </row>
@@ -1074,40 +1058,44 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>UHID-1015</t>
+          <t>UHID-1016</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Dr. Manish Gupta</t>
+          <t>Dr. Kavita Nair</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Orthopaedics</t>
+          <t>Neurology</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>08:15</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>booked</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Follow-up</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr"/>
+          <t>OPD</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Routine check-up</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1117,7 +1105,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>UHID-1010</t>
+          <t>UHID-1011</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1127,27 +1115,27 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Gynaecology</t>
+          <t>Paediatrics</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>cancelled</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Follow-up</t>
+          <t>Procedure</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1169,22 +1157,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Dr. Kavita Nair</t>
+          <t>Dr. Manish Gupta</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Gastroenterology</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>13:45</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1211,32 +1199,32 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>UHID-1018</t>
+          <t>UHID-1005</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Dr. Rajesh Kumar</t>
+          <t>Dr. Vikram Rao</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Orthopaedics</t>
+          <t>Gynaecology</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>booked</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1246,7 +1234,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Post-surgery review</t>
+          <t>Routine check-up</t>
         </is>
       </c>
     </row>
@@ -1258,17 +1246,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>UHID-1014</t>
+          <t>UHID-1016</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Dr. Arjun Verma</t>
+          <t>Dr. Kavita Nair</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Orthopaedics</t>
+          <t>Oncology</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1278,12 +1266,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>cancelled</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1291,7 +1279,11 @@
           <t>OPD</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Routine check-up</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1301,17 +1293,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>UHID-1001</t>
+          <t>UHID-1008</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Dr. Rajesh Kumar</t>
+          <t>Dr. Kavita Nair</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Neurology</t>
+          <t>Pulmonology</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1321,12 +1313,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>booked</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1334,7 +1326,11 @@
           <t>Procedure</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Post-surgery review</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1349,37 +1345,37 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Dr. Sunita Sharma</t>
+          <t>Dr. Priya Mehta</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Orthopaedics</t>
+          <t>Psychiatry</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>booked</t>
+          <t>cancelled</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Review</t>
+          <t>Procedure</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Routine check-up</t>
+          <t>Medication review</t>
         </is>
       </c>
     </row>
@@ -1396,27 +1392,27 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Dr. Rajesh Kumar</t>
+          <t>Dr. Deepa Iyer</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Nephrology</t>
+          <t>Orthopaedics</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>11:15</t>
+          <t>16:15</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>cancelled</t>
+          <t>booked</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1424,11 +1420,7 @@
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>Post-surgery review</t>
-        </is>
-      </c>
+      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1438,42 +1430,42 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>UHID-1019</t>
+          <t>UHID-1009</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Dr. Rajesh Kumar</t>
+          <t>Dr. Suresh Reddy</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Nephrology</t>
+          <t>Oncology</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>cancelled</t>
+          <t>booked</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>OPD</t>
+          <t>Procedure</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Routine check-up</t>
+          <t>Medication review</t>
         </is>
       </c>
     </row>
@@ -1485,27 +1477,27 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>UHID-1002</t>
+          <t>UHID-1010</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Dr. Arjun Verma</t>
+          <t>Dr. Vikram Rao</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Orthopaedics</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1515,14 +1507,10 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Follow-up</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>Post-surgery review</t>
-        </is>
-      </c>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1532,12 +1520,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>UHID-1016</t>
+          <t>UHID-1002</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Dr. Arjun Verma</t>
+          <t>Dr. Priya Mehta</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1547,7 +1535,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1562,10 +1550,14 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr"/>
+          <t>Follow-up</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Routine check-up</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1575,17 +1567,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>UHID-1003</t>
+          <t>UHID-1004</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Dr. Arjun Verma</t>
+          <t>Dr. Priya Mehta</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Gastroenterology</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1595,7 +1587,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1605,7 +1597,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Review</t>
+          <t>Procedure</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1622,27 +1614,27 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>UHID-1009</t>
+          <t>UHID-1012</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Dr. Kavita Nair</t>
+          <t>Dr. Anita Singh</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Nephrology</t>
+          <t>Oncology</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>09:15</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1652,10 +1644,14 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Follow-up</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr"/>
+          <t>Procedure</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Medication review</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1665,27 +1661,27 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>UHID-1014</t>
+          <t>UHID-1017</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Dr. Suresh Reddy</t>
+          <t>Dr. Manish Gupta</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Orthopaedics</t>
+          <t>Paediatrics</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1695,7 +1691,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Review</t>
+          <t>Follow-up</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1712,27 +1708,27 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>UHID-1016</t>
+          <t>UHID-1018</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Dr. Sunita Sharma</t>
+          <t>Dr. Deepa Iyer</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Paediatrics</t>
+          <t>Nephrology</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1742,7 +1738,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Follow-up</t>
+          <t>Procedure</t>
         </is>
       </c>
       <c r="I29" t="inlineStr"/>
@@ -1755,12 +1751,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>UHID-1015</t>
+          <t>UHID-1016</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Dr. Arjun Verma</t>
+          <t>Dr. Manish Gupta</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1770,29 +1766,25 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>13:45</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>booked</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>OPD</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>Medication review</t>
-        </is>
-      </c>
+          <t>Follow-up</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1802,32 +1794,32 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>UHID-1010</t>
+          <t>UHID-1012</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Dr. Deepa Iyer</t>
+          <t>Dr. Kavita Nair</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Orthopaedics</t>
+          <t>Pulmonology</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>cancelled</t>
+          <t>booked</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1837,7 +1829,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Post-surgery review</t>
+          <t>Routine check-up</t>
         </is>
       </c>
     </row>

</xml_diff>